<commit_message>
Integrated more pages from backend-main branch
</commit_message>
<xml_diff>
--- a/kickback-docs/KickBack_ExcelSheet.xlsx
+++ b/kickback-docs/KickBack_ExcelSheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30306"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/88d804889d8adff9/Desktop/KIckback/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/88d804889d8adff9/Desktop/KickBack/kickback-docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B624294C-E802-41B8-83D5-CF1EA36E69C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{B624294C-E802-41B8-83D5-CF1EA36E69C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0689686-6DD0-40A7-BC5A-1B4663FAFFAE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{4911757A-3624-4C7A-81A1-7FBB81A1AAD3}"/>
   </bookViews>
@@ -35,15 +35,379 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>KickBack Backend — Round 2 Fixes</t>
+  </si>
+  <si>
+    <t>1. Double-booking race condition — not yet fixed (highest priority)</t>
+  </si>
+  <si>
+    <r>
+      <t>BookingService.createBooking()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> checks </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>existsOverlappingBooking()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and then inserts, but nothing locks the resource between the check and the insert. Two simultaneous requests for the same slot can both pass the check and both succeed.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Fix: before the overlap check, acquire a pessimistic write lock on the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Resource</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> row being booked (e.g. a repository method annotated </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>@Lock(LockModeType.PESSIMISTIC_WRITE)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> that fetches the resource by ID). This serializes all booking attempts for that resource, so the overlap check and insert that follow are guaranteed race-free — regardless of how the overlap query itself is written.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>isClosedToday</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>isActive</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — still not fixed</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Same fields as before, still missing </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>@JsonProperty("isClosedToday")</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> on </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>OperatingWindowResponse</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>@JsonProperty("isActive")</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> on </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>OfferSummaryResponse</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. No changes were made here yet.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>avatar_id</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — still not added</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">No column on </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>User</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, no field on </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>UserProfileResponse</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>UpdateProfileRequest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Still pending.</t>
+    </r>
+  </si>
+  <si>
+    <t>4. Missing: a "list my bookings" endpoint</t>
+  </si>
+  <si>
+    <r>
+      <t>BookingController</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> has </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>GET /bookings/{id}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (single) but nothing to list a user's bookings (e.g. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>GET /users/me/bookings</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>). Needed for the My Bookings screen.</t>
+    </r>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -66,8 +430,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,9 +778,75 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A3B8726-437A-4C20-8198-F51BCB8D623B}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
-  <sheetData/>
+  <dimension ref="A1:A18"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="112.33203125" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="2"/>
+    </row>
+    <row r="5" spans="1:1" ht="28.8">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="43.2">
+      <c r="A6" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="2"/>
+    </row>
+    <row r="10" spans="1:1" ht="28.8">
+      <c r="A10" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="2"/>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="2"/>
+    </row>
+    <row r="18" spans="1:1" ht="28.8">
+      <c r="A18" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>